<commit_message>
Zmysl dane przykladowe, odswiez pule pytan, opisz zasoby Media
- Team Members i autorzy recenzji: nazwiska zastapione fikcyjnymi,
  zeby w publicznym repo nie bylo danych prawdziwych osob.
- Pula pytan rozszerzona do 72 pozycji w pieciu kategoriach,
  czesc zainspirowana typowymi listami icebreakerow.
- Nowe katalogi media/ w obu aplikacjach: tabela mapowania
  plik -> nazwa zasobu -> kontrolka, instrukcja podpiecia w Studio
  i sposob wyciagniecia plikow z istniejacej aplikacji (.msapp).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HuZ5btZPoBe1uBra3QrvBc
</commit_message>
<xml_diff>
--- a/powerapps/kartoteka/sharepoint/Recenzje.xlsx
+++ b/powerapps/kartoteka/sharepoint/Recenzje.xlsx
@@ -483,7 +483,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Romanowski Piotr</t>
+          <t>Pierogowska Anna</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Klein Ewa</t>
+          <t>Kompotowski Bartosz</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Gwiazda Marcin</t>
+          <t>Żurkiewicz Celina</t>
         </is>
       </c>
     </row>
@@ -554,7 +554,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Adamczyk Natalia</t>
+          <t>Makowiecki Damian</t>
         </is>
       </c>
     </row>
@@ -579,7 +579,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Borowiec Tomasz</t>
+          <t>Rogalik Emilia</t>
         </is>
       </c>
     </row>
@@ -604,7 +604,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Cieślak Magdalena</t>
+          <t>Barszczyński Fabian</t>
         </is>
       </c>
     </row>
@@ -629,7 +629,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Dąbrowski Rafał</t>
+          <t>Kluskowska Gabriela</t>
         </is>
       </c>
     </row>
@@ -654,7 +654,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Fijałkowska Iwona</t>
+          <t>Serowacki Henryk</t>
         </is>
       </c>
     </row>
@@ -679,7 +679,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Grabowski Michał</t>
+          <t>Naleśnikowska Iwona</t>
         </is>
       </c>
     </row>
@@ -704,7 +704,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Herman Alicja</t>
+          <t>Ogórecki Jakub</t>
         </is>
       </c>
     </row>
@@ -729,7 +729,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Jankowski Paweł</t>
+          <t>Truskawiecka Kamila</t>
         </is>
       </c>
     </row>
@@ -754,7 +754,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Kowalczyk Dorota</t>
+          <t>Piernikowski Leon</t>
         </is>
       </c>
     </row>
@@ -779,7 +779,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Lewandowska Karolina</t>
+          <t>Sernikowska Marta</t>
         </is>
       </c>
     </row>
@@ -804,7 +804,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Maj Sebastian</t>
+          <t>Bigosiewicz Norbert</t>
         </is>
       </c>
     </row>
@@ -829,7 +829,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Nowicki Adam</t>
+          <t>Śliwkowska Olga</t>
         </is>
       </c>
     </row>
@@ -850,7 +850,7 @@
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Ostrowska Joanna</t>
+          <t>Grzybowiecki Patryk</t>
         </is>
       </c>
     </row>
@@ -875,7 +875,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Pawlak Krzysztof</t>
+          <t>Pyzowska Renata</t>
         </is>
       </c>
     </row>
@@ -900,7 +900,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Rutkowska Beata</t>
+          <t>Zapiekanko Sebastian</t>
         </is>
       </c>
     </row>
@@ -925,7 +925,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Sikora Damian</t>
+          <t>Placuszek Weronika</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Wójcik Anna</t>
+          <t>Chałkowski Zbigniew</t>
         </is>
       </c>
     </row>

</xml_diff>